<commit_message>
Fixed graph scaling in section 1
</commit_message>
<xml_diff>
--- a/data/02-processed/caces_state_year.xlsx
+++ b/data/02-processed/caces_state_year.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47420,7 +47420,7 @@
         <v>17.93956447003103</v>
       </c>
       <c r="G1818" t="n">
-        <v>7.161047621647617</v>
+        <v>7.161047621647618</v>
       </c>
       <c r="H1818" t="n">
         <v>0.7716176000147071</v>
@@ -47448,7 +47448,7 @@
         <v>15.44731635706157</v>
       </c>
       <c r="G1819" t="n">
-        <v>4.209671305696958</v>
+        <v>4.209671305696959</v>
       </c>
       <c r="H1819" t="n">
         <v>0.9834606966822154</v>
@@ -47554,7 +47554,7 @@
         <v>2.999216943828253</v>
       </c>
       <c r="E1823" t="n">
-        <v>35.918543588158</v>
+        <v>35.91854358815801</v>
       </c>
       <c r="F1823" t="n">
         <v>13.4199062023167</v>
@@ -47750,7 +47750,7 @@
         <v>2.782665100625103</v>
       </c>
       <c r="E1830" t="n">
-        <v>42.56752760665963</v>
+        <v>42.56752760665964</v>
       </c>
       <c r="F1830" t="n">
         <v>12.64782952722966</v>
@@ -48055,7 +48055,7 @@
         <v>0.1793945761332227</v>
       </c>
       <c r="D1841" t="n">
-        <v>2.999293561821394</v>
+        <v>2.999293561821395</v>
       </c>
       <c r="E1841" t="n">
         <v>36.12161084522987</v>
@@ -48506,7 +48506,7 @@
         <v>4.002766507710818</v>
       </c>
       <c r="E1857" t="n">
-        <v>50.09369507200399</v>
+        <v>50.093695072004</v>
       </c>
       <c r="F1857" t="n">
         <v>13.68179464594462</v>
@@ -48596,7 +48596,7 @@
         <v>11.76652406299505</v>
       </c>
       <c r="G1860" t="n">
-        <v>5.233957763896849</v>
+        <v>5.23395776389685</v>
       </c>
       <c r="H1860" t="n">
         <v>1.00091518658981</v>
@@ -48615,7 +48615,7 @@
         <v>0.1668887305150394</v>
       </c>
       <c r="D1861" t="n">
-        <v>3.449798948256143</v>
+        <v>3.449798948256144</v>
       </c>
       <c r="E1861" t="n">
         <v>37.9451930505962</v>
@@ -48848,7 +48848,7 @@
         <v>9.401982116057042</v>
       </c>
       <c r="G1869" t="n">
-        <v>5.388840579949116</v>
+        <v>5.388840579949117</v>
       </c>
       <c r="H1869" t="n">
         <v>0.6600992222111275</v>
@@ -48926,7 +48926,7 @@
         <v>2.768539442401414</v>
       </c>
       <c r="E1872" t="n">
-        <v>33.55042565639615</v>
+        <v>33.55042565639616</v>
       </c>
       <c r="F1872" t="n">
         <v>13.87048255022058</v>
@@ -49016,7 +49016,7 @@
         <v>14.43553049636949</v>
       </c>
       <c r="G1875" t="n">
-        <v>7.58147949325835</v>
+        <v>7.581479493258351</v>
       </c>
       <c r="H1875" t="n">
         <v>1.056980912419028</v>
@@ -49035,10 +49035,10 @@
         <v>0.1758577708014357</v>
       </c>
       <c r="D1876" t="n">
-        <v>4.029237548952214</v>
+        <v>4.029237548952215</v>
       </c>
       <c r="E1876" t="n">
-        <v>45.27379645874854</v>
+        <v>45.27379645874855</v>
       </c>
       <c r="F1876" t="n">
         <v>18.59749831304817</v>
@@ -49293,7 +49293,7 @@
         <v>37.9929647667914</v>
       </c>
       <c r="F1885" t="n">
-        <v>18.89506297966396</v>
+        <v>18.89506297966397</v>
       </c>
       <c r="G1885" t="n">
         <v>5.940207581412438</v>
@@ -49315,7 +49315,7 @@
         <v>0.1995268850432412</v>
       </c>
       <c r="D1886" t="n">
-        <v>3.017106633680279</v>
+        <v>3.01710663368028</v>
       </c>
       <c r="E1886" t="n">
         <v>44.08986263492864</v>
@@ -49430,7 +49430,7 @@
         <v>2.84725794547816</v>
       </c>
       <c r="E1890" t="n">
-        <v>39.45669041295002</v>
+        <v>39.45669041295004</v>
       </c>
       <c r="F1890" t="n">
         <v>18.00226285348845</v>
@@ -49906,7 +49906,7 @@
         <v>3.4708638118368</v>
       </c>
       <c r="E1907" t="n">
-        <v>41.22463047222578</v>
+        <v>41.22463047222579</v>
       </c>
       <c r="F1907" t="n">
         <v>10.81337179170983</v>
@@ -49990,7 +49990,7 @@
         <v>3.034577910779488</v>
       </c>
       <c r="E1910" t="n">
-        <v>39.32501661391616</v>
+        <v>39.32501661391617</v>
       </c>
       <c r="F1910" t="n">
         <v>14.85860641522944</v>
@@ -50018,7 +50018,7 @@
         <v>2.755064220668803</v>
       </c>
       <c r="E1911" t="n">
-        <v>40.42238317265834</v>
+        <v>40.42238317265835</v>
       </c>
       <c r="F1911" t="n">
         <v>10.47372336595036</v>
@@ -50214,7 +50214,7 @@
         <v>5.543381440485197</v>
       </c>
       <c r="E1918" t="n">
-        <v>39.87742506278861</v>
+        <v>39.87742506278862</v>
       </c>
       <c r="F1918" t="n">
         <v>10.34338021957163</v>
@@ -50304,7 +50304,7 @@
         <v>15.34055817797867</v>
       </c>
       <c r="G1921" t="n">
-        <v>6.506616791196091</v>
+        <v>6.506616791196092</v>
       </c>
       <c r="H1921" t="n">
         <v>0.6824419072655649</v>
@@ -50528,7 +50528,7 @@
         <v>15.54841205809331</v>
       </c>
       <c r="G1929" t="n">
-        <v>7.711848508750285</v>
+        <v>7.711848508750284</v>
       </c>
       <c r="H1929" t="n">
         <v>0.7167474226741462</v>
@@ -50746,7 +50746,7 @@
         <v>3.362845420389253</v>
       </c>
       <c r="E1937" t="n">
-        <v>42.53952228785281</v>
+        <v>42.53952228785282</v>
       </c>
       <c r="F1937" t="n">
         <v>12.46250589302171</v>
@@ -51191,7 +51191,7 @@
         <v>0.1893445412602272</v>
       </c>
       <c r="D1953" t="n">
-        <v>2.627547838095621</v>
+        <v>2.62754783809562</v>
       </c>
       <c r="E1953" t="n">
         <v>40.77363376677028</v>
@@ -51919,7 +51919,7 @@
         <v>0.1966289237082255</v>
       </c>
       <c r="D1979" t="n">
-        <v>5.10670156582577</v>
+        <v>5.106701565825771</v>
       </c>
       <c r="E1979" t="n">
         <v>38.26387509693591</v>
@@ -52006,7 +52006,7 @@
         <v>3.525650896016225</v>
       </c>
       <c r="E1982" t="n">
-        <v>37.38644320368883</v>
+        <v>37.38644320368884</v>
       </c>
       <c r="F1982" t="n">
         <v>11.11234422991702</v>
@@ -52681,7 +52681,7 @@
         <v>34.18420072220055</v>
       </c>
       <c r="F2006" t="n">
-        <v>7.661110473515241</v>
+        <v>7.661110473515242</v>
       </c>
       <c r="G2006" t="n">
         <v>3.849982852830558</v>
@@ -52822,7 +52822,7 @@
         <v>10.91747409011333</v>
       </c>
       <c r="G2011" t="n">
-        <v>6.446889018427168</v>
+        <v>6.446889018427169</v>
       </c>
       <c r="H2011" t="n">
         <v>0.5183141517468595</v>
@@ -52919,7 +52919,7 @@
         <v>0.1939993283557542</v>
       </c>
       <c r="D2015" t="n">
-        <v>3.672324474163189</v>
+        <v>3.67232447416319</v>
       </c>
       <c r="E2015" t="inlineStr"/>
       <c r="F2015" t="n">
@@ -53391,7 +53391,7 @@
       </c>
       <c r="E2033" t="inlineStr"/>
       <c r="F2033" t="n">
-        <v>15.16017080062654</v>
+        <v>15.16017080062655</v>
       </c>
       <c r="G2033" t="n">
         <v>6.626205617823736</v>
@@ -53472,7 +53472,7 @@
         <v>9.105041974935057</v>
       </c>
       <c r="G2036" t="n">
-        <v>5.450792642454005</v>
+        <v>5.450792642454006</v>
       </c>
       <c r="H2036" t="n">
         <v>0.4664631959888794</v>
@@ -53576,7 +53576,7 @@
         <v>12.23523561772947</v>
       </c>
       <c r="G2040" t="n">
-        <v>6.316533742654197</v>
+        <v>6.316533742654198</v>
       </c>
       <c r="H2040" t="n">
         <v>0.3695743401254863</v>
@@ -53907,7 +53907,7 @@
         <v>0.1918863718624545</v>
       </c>
       <c r="D2053" t="n">
-        <v>4.537098597404095</v>
+        <v>4.537098597404094</v>
       </c>
       <c r="E2053" t="inlineStr"/>
       <c r="F2053" t="n">
@@ -54037,7 +54037,7 @@
         <v>0.1679546816459772</v>
       </c>
       <c r="D2058" t="n">
-        <v>2.661925994798188</v>
+        <v>2.661925994798187</v>
       </c>
       <c r="E2058" t="inlineStr"/>
       <c r="F2058" t="n">

</xml_diff>

<commit_message>
Analysis, removed bulk from eda
</commit_message>
<xml_diff>
--- a/data/02-processed/caces_state_year.xlsx
+++ b/data/02-processed/caces_state_year.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47420,7 +47420,7 @@
         <v>17.93956447003103</v>
       </c>
       <c r="G1818" t="n">
-        <v>7.161047621647618</v>
+        <v>7.161047621647617</v>
       </c>
       <c r="H1818" t="n">
         <v>0.7716176000147071</v>
@@ -47448,7 +47448,7 @@
         <v>15.44731635706157</v>
       </c>
       <c r="G1819" t="n">
-        <v>4.209671305696959</v>
+        <v>4.209671305696958</v>
       </c>
       <c r="H1819" t="n">
         <v>0.9834606966822154</v>
@@ -47554,7 +47554,7 @@
         <v>2.999216943828253</v>
       </c>
       <c r="E1823" t="n">
-        <v>35.91854358815801</v>
+        <v>35.918543588158</v>
       </c>
       <c r="F1823" t="n">
         <v>13.4199062023167</v>
@@ -47750,7 +47750,7 @@
         <v>2.782665100625103</v>
       </c>
       <c r="E1830" t="n">
-        <v>42.56752760665964</v>
+        <v>42.56752760665963</v>
       </c>
       <c r="F1830" t="n">
         <v>12.64782952722966</v>
@@ -48055,7 +48055,7 @@
         <v>0.1793945761332227</v>
       </c>
       <c r="D1841" t="n">
-        <v>2.999293561821395</v>
+        <v>2.999293561821394</v>
       </c>
       <c r="E1841" t="n">
         <v>36.12161084522987</v>
@@ -48506,7 +48506,7 @@
         <v>4.002766507710818</v>
       </c>
       <c r="E1857" t="n">
-        <v>50.093695072004</v>
+        <v>50.09369507200399</v>
       </c>
       <c r="F1857" t="n">
         <v>13.68179464594462</v>
@@ -48596,7 +48596,7 @@
         <v>11.76652406299505</v>
       </c>
       <c r="G1860" t="n">
-        <v>5.23395776389685</v>
+        <v>5.233957763896849</v>
       </c>
       <c r="H1860" t="n">
         <v>1.00091518658981</v>
@@ -48615,7 +48615,7 @@
         <v>0.1668887305150394</v>
       </c>
       <c r="D1861" t="n">
-        <v>3.449798948256144</v>
+        <v>3.449798948256143</v>
       </c>
       <c r="E1861" t="n">
         <v>37.9451930505962</v>
@@ -48848,7 +48848,7 @@
         <v>9.401982116057042</v>
       </c>
       <c r="G1869" t="n">
-        <v>5.388840579949117</v>
+        <v>5.388840579949116</v>
       </c>
       <c r="H1869" t="n">
         <v>0.6600992222111275</v>
@@ -48926,7 +48926,7 @@
         <v>2.768539442401414</v>
       </c>
       <c r="E1872" t="n">
-        <v>33.55042565639616</v>
+        <v>33.55042565639615</v>
       </c>
       <c r="F1872" t="n">
         <v>13.87048255022058</v>
@@ -49016,7 +49016,7 @@
         <v>14.43553049636949</v>
       </c>
       <c r="G1875" t="n">
-        <v>7.581479493258351</v>
+        <v>7.58147949325835</v>
       </c>
       <c r="H1875" t="n">
         <v>1.056980912419028</v>
@@ -49035,10 +49035,10 @@
         <v>0.1758577708014357</v>
       </c>
       <c r="D1876" t="n">
-        <v>4.029237548952215</v>
+        <v>4.029237548952214</v>
       </c>
       <c r="E1876" t="n">
-        <v>45.27379645874855</v>
+        <v>45.27379645874854</v>
       </c>
       <c r="F1876" t="n">
         <v>18.59749831304817</v>
@@ -49293,7 +49293,7 @@
         <v>37.9929647667914</v>
       </c>
       <c r="F1885" t="n">
-        <v>18.89506297966397</v>
+        <v>18.89506297966396</v>
       </c>
       <c r="G1885" t="n">
         <v>5.940207581412438</v>
@@ -49315,7 +49315,7 @@
         <v>0.1995268850432412</v>
       </c>
       <c r="D1886" t="n">
-        <v>3.01710663368028</v>
+        <v>3.017106633680279</v>
       </c>
       <c r="E1886" t="n">
         <v>44.08986263492864</v>
@@ -49430,7 +49430,7 @@
         <v>2.84725794547816</v>
       </c>
       <c r="E1890" t="n">
-        <v>39.45669041295004</v>
+        <v>39.45669041295002</v>
       </c>
       <c r="F1890" t="n">
         <v>18.00226285348845</v>
@@ -49906,7 +49906,7 @@
         <v>3.4708638118368</v>
       </c>
       <c r="E1907" t="n">
-        <v>41.22463047222579</v>
+        <v>41.22463047222578</v>
       </c>
       <c r="F1907" t="n">
         <v>10.81337179170983</v>
@@ -49990,7 +49990,7 @@
         <v>3.034577910779488</v>
       </c>
       <c r="E1910" t="n">
-        <v>39.32501661391617</v>
+        <v>39.32501661391616</v>
       </c>
       <c r="F1910" t="n">
         <v>14.85860641522944</v>
@@ -50018,7 +50018,7 @@
         <v>2.755064220668803</v>
       </c>
       <c r="E1911" t="n">
-        <v>40.42238317265835</v>
+        <v>40.42238317265834</v>
       </c>
       <c r="F1911" t="n">
         <v>10.47372336595036</v>
@@ -50214,7 +50214,7 @@
         <v>5.543381440485197</v>
       </c>
       <c r="E1918" t="n">
-        <v>39.87742506278862</v>
+        <v>39.87742506278861</v>
       </c>
       <c r="F1918" t="n">
         <v>10.34338021957163</v>
@@ -50304,7 +50304,7 @@
         <v>15.34055817797867</v>
       </c>
       <c r="G1921" t="n">
-        <v>6.506616791196092</v>
+        <v>6.506616791196091</v>
       </c>
       <c r="H1921" t="n">
         <v>0.6824419072655649</v>
@@ -50528,7 +50528,7 @@
         <v>15.54841205809331</v>
       </c>
       <c r="G1929" t="n">
-        <v>7.711848508750284</v>
+        <v>7.711848508750285</v>
       </c>
       <c r="H1929" t="n">
         <v>0.7167474226741462</v>
@@ -50746,7 +50746,7 @@
         <v>3.362845420389253</v>
       </c>
       <c r="E1937" t="n">
-        <v>42.53952228785282</v>
+        <v>42.53952228785281</v>
       </c>
       <c r="F1937" t="n">
         <v>12.46250589302171</v>
@@ -51191,7 +51191,7 @@
         <v>0.1893445412602272</v>
       </c>
       <c r="D1953" t="n">
-        <v>2.62754783809562</v>
+        <v>2.627547838095621</v>
       </c>
       <c r="E1953" t="n">
         <v>40.77363376677028</v>
@@ -51919,7 +51919,7 @@
         <v>0.1966289237082255</v>
       </c>
       <c r="D1979" t="n">
-        <v>5.106701565825771</v>
+        <v>5.10670156582577</v>
       </c>
       <c r="E1979" t="n">
         <v>38.26387509693591</v>
@@ -52006,7 +52006,7 @@
         <v>3.525650896016225</v>
       </c>
       <c r="E1982" t="n">
-        <v>37.38644320368884</v>
+        <v>37.38644320368883</v>
       </c>
       <c r="F1982" t="n">
         <v>11.11234422991702</v>
@@ -52681,7 +52681,7 @@
         <v>34.18420072220055</v>
       </c>
       <c r="F2006" t="n">
-        <v>7.661110473515242</v>
+        <v>7.661110473515241</v>
       </c>
       <c r="G2006" t="n">
         <v>3.849982852830558</v>
@@ -52822,7 +52822,7 @@
         <v>10.91747409011333</v>
       </c>
       <c r="G2011" t="n">
-        <v>6.446889018427169</v>
+        <v>6.446889018427168</v>
       </c>
       <c r="H2011" t="n">
         <v>0.5183141517468595</v>
@@ -52919,7 +52919,7 @@
         <v>0.1939993283557542</v>
       </c>
       <c r="D2015" t="n">
-        <v>3.67232447416319</v>
+        <v>3.672324474163189</v>
       </c>
       <c r="E2015" t="inlineStr"/>
       <c r="F2015" t="n">
@@ -53391,7 +53391,7 @@
       </c>
       <c r="E2033" t="inlineStr"/>
       <c r="F2033" t="n">
-        <v>15.16017080062655</v>
+        <v>15.16017080062654</v>
       </c>
       <c r="G2033" t="n">
         <v>6.626205617823736</v>
@@ -53472,7 +53472,7 @@
         <v>9.105041974935057</v>
       </c>
       <c r="G2036" t="n">
-        <v>5.450792642454006</v>
+        <v>5.450792642454005</v>
       </c>
       <c r="H2036" t="n">
         <v>0.4664631959888794</v>
@@ -53576,7 +53576,7 @@
         <v>12.23523561772947</v>
       </c>
       <c r="G2040" t="n">
-        <v>6.316533742654198</v>
+        <v>6.316533742654197</v>
       </c>
       <c r="H2040" t="n">
         <v>0.3695743401254863</v>
@@ -53907,7 +53907,7 @@
         <v>0.1918863718624545</v>
       </c>
       <c r="D2053" t="n">
-        <v>4.537098597404094</v>
+        <v>4.537098597404095</v>
       </c>
       <c r="E2053" t="inlineStr"/>
       <c r="F2053" t="n">
@@ -54037,7 +54037,7 @@
         <v>0.1679546816459772</v>
       </c>
       <c r="D2058" t="n">
-        <v>2.661925994798187</v>
+        <v>2.661925994798188</v>
       </c>
       <c r="E2058" t="inlineStr"/>
       <c r="F2058" t="n">

</xml_diff>